<commit_message>
Software requirements specification, and seven more UAT scenarios
srs/srs.md follows the structure of github.com/jam01/SRS-Template: 79 requirements, each with an ID, a
statement, a rationale, acceptance criteria and a verification method, generated from the state model and
the working papers by srs/build_srs.py. Seven scenarios added for the riskiest untested moves (54 in all);
46 of the 63 moves in the transition table now have a UAT scenario.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/uat/uat-script.xlsx
+++ b/uat/uat-script.xlsx
@@ -173,8 +173,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UAT" displayName="UAT" ref="A1:N48" headerRowCount="1">
-  <autoFilter ref="A1:N48"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UAT" displayName="UAT" ref="A1:N55" headerRowCount="1">
+  <autoFilter ref="A1:N55"/>
   <tableColumns count="14">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Story"/>
@@ -623,7 +623,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Refused moves in the model that no row tests: delivery-trip, Delivered: edit times or quantities; delivery-trip, Planned: edit when the order is closed; sales-order, Completed: edit; sales-order, Receiving and shipping: cancel. A choice, not a gap: each is enforced by the same rule as a tested move.</t>
+          <t>Refused moves in the model that no row tests: delivery-trip, Planned: edit when the order is closed. A choice, not a gap: each is enforced by the same rule as a tested move.</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N48"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1169,40 +1169,104 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>delivery-trip</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>A delivered trip's times and quantities cannot be edited</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>delivery-trip</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>refused in Delivered: edit times or quantities</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>T10, T16, T11, T17</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>D14, D15, D16</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Given order "SO-2050" is "Receiving and shipping"
+And trip "TR-118" is planned to deliver 5 of "Container C-20" for it
+Given trip "TR-118" is "Delivered"
+When the logistics coordinator tries to change its delivered quantity to 4</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Then the change is refused
+And the logistics coordinator sees "A delivered trip is read-only."</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr"/>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Logistics coordinator</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>UAT-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
           <t>material-request</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>A numbered issue form cannot exist before the materials are issued</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>material-request</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>refused in Open: download numbered form</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>T7</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>D6, D15</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2070" for 300 steel drums is "In production"
 And material request "MR-310" for it asks for 400 kg of "Steel sheet 1.2 mm"
@@ -1211,63 +1275,63 @@
 When the warehouse keeper tries to download the numbered issue form</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Then the download is refused
 And the warehouse keeper sees "No stock has moved yet. Preview the draft form; its number is given when the materials are issued."</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="3" t="inlineStr">
         <is>
           <t>Warehouse keeper</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>UAT-08</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="N9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>UAT-09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>material-request</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>The first issue starts the request</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>material-request</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Open: issue first materials, to Issuing</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>T7</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>D6, D15</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2070" for 300 steel drums is "In production"
 And material request "MR-310" for it asks for 400 kg of "Steel sheet 1.2 mm"
@@ -1276,64 +1340,64 @@
 When the warehouse keeper issues 250 kg to the drum workshop</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Then "MR-310" shows the state "Issuing"
 And stock of "Steel sheet 1.2 mm" falls by 250 kg
 And the issue form downloads with its form number</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr">
         <is>
           <t>Warehouse keeper</t>
         </is>
       </c>
-      <c r="N9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>UAT-09</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="N10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>UAT-10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>material-request</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>A second issue gets its own form</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>material-request</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Issuing: issue more materials, to Issuing</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>T4, T7</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>D6, D15</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2070" for 300 steel drums is "In production"
 And material request "MR-310" for it asks for 400 kg of "Steel sheet 1.2 mm"
@@ -1342,63 +1406,63 @@
 When the warehouse keeper issues 100 kg to the drum workshop</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Then "MR-310" still shows the state "Issuing"
 And a new issue form downloads with its own form number</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr"/>
-      <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr"/>
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>Warehouse keeper</t>
         </is>
       </c>
-      <c r="N10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>UAT-10</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>UAT-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>material-request</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>The last issue completes the request</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>material-request</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Issuing: issue last materials, to Completed</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>T4, T7</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>D6, D15</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2070" for 300 steel drums is "In production"
 And material request "MR-310" for it asks for 400 kg of "Steel sheet 1.2 mm"
@@ -1407,62 +1471,62 @@
 When the warehouse keeper issues the last 50 kg</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Then "MR-310" shows the state "Completed"</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr"/>
-      <c r="L11" s="3" t="inlineStr"/>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr"/>
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>Warehouse keeper</t>
         </is>
       </c>
-      <c r="N11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>UAT-11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="N12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>UAT-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>material-request</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>A request that has issued materials cannot be cancelled</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>material-request</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>refused in Issuing: cancel</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>T4, T7</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>D6, D15</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2070" for 300 steel drums is "In production"
 And material request "MR-310" for it asks for 400 kg of "Steel sheet 1.2 mm"
@@ -1471,63 +1535,63 @@
 When the factory manager tries to cancel it</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Then the cancellation is refused
 And the factory manager sees "Materials have left the warehouse. Complete the request, or close the order as Not completed."</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr"/>
-      <c r="L12" s="3" t="inlineStr"/>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr"/>
+      <c r="M13" s="3" t="inlineStr">
         <is>
           <t>Factory manager</t>
         </is>
       </c>
-      <c r="N12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>UAT-12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="N13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>UAT-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>material-request</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>A request with nothing issued can be cancelled, and is kept</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>material-request</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Open: cancel, to Cancelled</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>T4, T7</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>D6, D15</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2070" for 300 steel drums is "In production"
 And material request "MR-310" for it asks for 400 kg of "Steel sheet 1.2 mm"
@@ -1536,79 +1600,17 @@
 When the factory manager cancels it</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Then "MR-311" shows the state "Cancelled"
 And it keeps its number</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr">
-        <is>
-          <t>Factory manager</t>
-        </is>
-      </c>
-      <c r="N13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>UAT-13</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>order-closure</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>An open order can be cancelled</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>sales-order</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Open: cancel, to Cancelled</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>G0, T14, G3, T15</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>D6, D10</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>Given order "SO-2040" is "Open"
-When the sales manager cancels it</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Then it shows the state "Cancelled"
-And order "SO-2040" can still be found and read</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr"/>
       <c r="L14" s="3" t="inlineStr"/>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>Sales staff; Sales manager</t>
+          <t>Factory manager</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr"/>
@@ -1626,219 +1628,470 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
+          <t>An open order can be cancelled</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>sales-order</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Open: cancel, to Cancelled</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>G0, T14, G3, T15</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>D6, D10</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Given order "SO-2040" is "Open"
+When the sales manager cancels it</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Then it shows the state "Cancelled"
+And order "SO-2040" can still be found and read</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr"/>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>Sales staff; Sales manager</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>UAT-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>order-closure</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
           <t>An order in production closes as not completed</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>sales-order</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>In production: close as not completed, to Not completed</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>T15</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>D6, D10</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2041" is "In production"
 And 4 of its 10 tank bodies have been received into stock
 When the sales manager closes it as not completed</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Then it shows the state "Not completed"
 And the 4 received assemblies stay in stock
 And the 6 not yet made drop out of open demand</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr"/>
-      <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr"/>
+      <c r="M16" s="3" t="inlineStr">
         <is>
           <t>Sales manager</t>
         </is>
       </c>
-      <c r="N15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>UAT-15</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="N16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>UAT-16</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>order-closure</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Nothing is removed when an order closes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>sales-order</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>in state: Cancelled</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>G0, T14, G3, T15</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>D6, D10</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2040" is "Cancelled"
 When anyone searches for order "SO-2040"</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Then the order is found with its history</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr"/>
-      <c r="L16" s="3" t="inlineStr"/>
-      <c r="M16" s="3" t="inlineStr"/>
-      <c r="N16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>UAT-16</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr"/>
+      <c r="M17" s="3" t="inlineStr"/>
+      <c r="N17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>UAT-17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>order-closure</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>An order in production cannot be cancelled</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>sales-order</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>refused in In production: cancel</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>T15, T9</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>D6, D10</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2041" is "In production"
 When the sales manager tries to cancel it</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>Then the cancellation is refused
 And the sales manager sees "Production has started. Close the order as Not completed instead."
 And order "SO-2041" still shows the state "In production"</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr"/>
+      <c r="L18" s="3" t="inlineStr"/>
+      <c r="M18" s="3" t="inlineStr">
         <is>
           <t>Sales manager</t>
         </is>
       </c>
-      <c r="N17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>UAT-17</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="N18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>UAT-18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>order-closure</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>An order with goods already received closes as not completed</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>sales-order</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Receiving and shipping: close as not completed, to Not completed</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>G0, T14, G3, T15</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>D6, D10</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Given order "SO-2043" is "Receiving and shipping"
+And 6 of its 10 containers have been received and 2 have been delivered
+When the sales manager closes it as not completed</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Then it shows the state "Not completed"
+And the 4 received containers not yet delivered stay in stock
+And the 4 not yet made drop out of open demand</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr"/>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>Sales manager</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>UAT-19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>order-closure</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>An order with goods already received cannot be cancelled</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>sales-order</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>refused in Receiving and shipping: cancel</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>G0, T14, G3, T15</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>D6, D10</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Given order "SO-2043" is "Receiving and shipping"
+When the sales manager tries to cancel it</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Then the cancellation is refused
+And the sales manager sees "Goods exist. Close the order as Not completed instead."
+And order "SO-2043" still shows the state "Receiving and shipping"</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr"/>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Sales manager</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>UAT-20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>order-closure</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>A completed order cannot be edited</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>sales-order</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>refused in Completed: edit</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>G0, T14, G3, T15</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>D6, D10</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Given order "SO-2044" is "Completed"
+When the sales manager tries to change the quantity on its first line</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Then the change is refused
+And the sales manager sees "A completed order is frozen."</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr"/>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>Sales manager</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>UAT-21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>order-lifecycle</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>A saved request does not start fulfilment</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>sales-order</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>in state: Request</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>T2, T18</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>D5, D7, D17</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" is on file
 And "Steel drum D-200" is a product Tanmark sells
@@ -1846,59 +2099,59 @@
 When logistics opens its work list</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>Then the request is not on it
 And the request shows the state "Request"</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr"/>
-      <c r="L18" s="3" t="inlineStr"/>
-      <c r="M18" s="3" t="inlineStr"/>
-      <c r="N18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>UAT-18</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="K22" s="3" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr"/>
+      <c r="M22" s="3" t="inlineStr"/>
+      <c r="N22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>UAT-22</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>order-lifecycle</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Confirming the request makes it an order</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>sales-order</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>Request: confirm order, to Open</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>D5, D7, D17</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" is on file
 And "Steel drum D-200" is a product Tanmark sells
@@ -1906,63 +2159,63 @@
 When Sam confirms the order</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>Then it shows the state "Open"
 And it has an order number</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr"/>
-      <c r="L19" s="3" t="inlineStr"/>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="3" t="inlineStr">
         <is>
           <t>Sales staff</t>
         </is>
       </c>
-      <c r="N19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>UAT-19</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="N23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>UAT-23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>order-lifecycle</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>A customer on credit hold gets no new order</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>sales-order</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>refused in Request: confirm on credit hold</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>R10</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>T2, T18</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>D5, D7, D17</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" is on file
 And "Steel drum D-200" is a product Tanmark sells
@@ -1971,64 +2224,64 @@
 When Sam tries to confirm the order</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Then the confirmation is refused
 And Sam sees "The customer is over its credit limit or overdue. The chief accountant must release the order."
 And the request still shows the state "Request"</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr"/>
-      <c r="L20" s="3" t="inlineStr"/>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="K24" s="3" t="inlineStr"/>
+      <c r="L24" s="3" t="inlineStr"/>
+      <c r="M24" s="3" t="inlineStr">
         <is>
           <t>Sales staff</t>
         </is>
       </c>
-      <c r="N20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>UAT-20</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="N24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>UAT-24</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>order-lifecycle</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>The chief accountant releases one order, with a reason</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>sales-order</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Request: confirm with credit release, to Open</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>R10</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>D5, D7, D17</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" is on file
 And "Steel drum D-200" is a product Tanmark sells
@@ -2037,63 +2290,63 @@
 When the chief accountant releases the order with the reason "Overdue invoice paid today; transfer confirmed"</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Then it shows the state "Open"
 And the release is logged with the chief accountant's name and the reason</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr"/>
-      <c r="L21" s="3" t="inlineStr"/>
-      <c r="M21" s="3" t="inlineStr">
+      <c r="K25" s="3" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr"/>
+      <c r="M25" s="3" t="inlineStr">
         <is>
           <t>Chief accountant</t>
         </is>
       </c>
-      <c r="N21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>UAT-21</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="N25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>UAT-25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>order-lifecycle</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Sending the order to logistics locks it for sales</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>sales-order</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Open: send to logistics, to With logistics</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>D5, D7, D17</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" is on file
 And "Steel drum D-200" is a product Tanmark sells
@@ -2101,63 +2354,63 @@
 When Sam sends it to logistics</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Then it shows the state "With logistics"
 And the logistics coordinator sees it on the work list</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr"/>
-      <c r="L22" s="3" t="inlineStr"/>
-      <c r="M22" s="3" t="inlineStr">
+      <c r="K26" s="3" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr"/>
+      <c r="M26" s="3" t="inlineStr">
         <is>
           <t>Sales staff</t>
         </is>
       </c>
-      <c r="N22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>UAT-22</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="N26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>UAT-26</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>order-lifecycle</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Sales cannot edit an order that logistics has</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>sales-order</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>refused in With logistics: sales edit</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>T14, T4</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>D5, D7, D17</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" is on file
 And "Steel drum D-200" is a product Tanmark sells
@@ -2165,554 +2418,554 @@
 When Sam tries to change its quantity from 6 to 8</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>Then the change is refused
 And Sam sees "After handoff, sales cannot edit the order. Raise a new order for an increase."
 And order "SO-2031" still shows a quantity of 6</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr"/>
-      <c r="L23" s="3" t="inlineStr"/>
-      <c r="M23" s="3" t="inlineStr">
+      <c r="K27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr"/>
+      <c r="M27" s="3" t="inlineStr">
         <is>
           <t>Sales staff</t>
         </is>
       </c>
-      <c r="N23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>UAT-23</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="N27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>UAT-27</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>A new purchase order is open at once</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>in state: Open</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>T6</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>D9, D15</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>Given the buyer holds a signed paper request for 200 kg of "Stainless bar S-40"
 When the buyer creates purchase order "PO-5110" with supplier "V-07"</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>Then it shows the state "Open"
 And no approval task is created</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr"/>
-      <c r="L24" s="3" t="inlineStr"/>
-      <c r="M24" s="3" t="inlineStr"/>
-      <c r="N24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>UAT-24</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="K28" s="3" t="inlineStr"/>
+      <c r="L28" s="3" t="inlineStr"/>
+      <c r="M28" s="3" t="inlineStr"/>
+      <c r="N28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>UAT-28</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>The warehouse keeper reviews a draft receipt form before receiving</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>in state: Open</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>T6</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>D9, D15</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>Given purchase order "PO-5110" is "Open"
 When the warehouse keeper previews the receipt form</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>Then the form downloads marked "Draft" with no form number
 And purchase order "PO-5110" still shows the state "Open"</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr"/>
-      <c r="L25" s="3" t="inlineStr"/>
-      <c r="M25" s="3" t="inlineStr"/>
-      <c r="N25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>UAT-25</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="K29" s="3" t="inlineStr"/>
+      <c r="L29" s="3" t="inlineStr"/>
+      <c r="M29" s="3" t="inlineStr"/>
+      <c r="N29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>UAT-29</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>A numbered receipt form cannot exist before the goods are received</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>refused in Open: download numbered form</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>T6</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>D9, D15</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>Given purchase order "PO-5110" is "Open"
 When the warehouse keeper tries to download the numbered receipt form</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>Then the download is refused
 And the warehouse keeper sees "No stock has moved yet. Preview the draft form; its number is given when the goods are received."</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr"/>
-      <c r="L26" s="3" t="inlineStr"/>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="K30" s="3" t="inlineStr"/>
+      <c r="L30" s="3" t="inlineStr"/>
+      <c r="M30" s="3" t="inlineStr">
         <is>
           <t>Warehouse keeper</t>
         </is>
       </c>
-      <c r="N26" s="3" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>UAT-26</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="N30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>UAT-30</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Receiving the goods counts as approval</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Open: receive into stock, to Received</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>T6</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>D9, D15</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>Given purchase order "PO-5110" is "Open"
 When the warehouse keeper receives 200 kg into stock against it</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>Then it shows the state "Received"
 And stock of "Stainless bar S-40" rises by 200 kg
 And the receipt form downloads with its form number</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr"/>
-      <c r="L27" s="3" t="inlineStr"/>
-      <c r="M27" s="3" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr"/>
+      <c r="L31" s="3" t="inlineStr"/>
+      <c r="M31" s="3" t="inlineStr">
         <is>
           <t>Warehouse keeper</t>
         </is>
       </c>
-      <c r="N27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>UAT-27</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="N31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>UAT-31</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>A second delivery gets its own receipt form</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>Received: receive more, to Received</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>T5, T6</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>D9, D15</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>Given purchase order "PO-5120" for 300 kg of "Stainless bar S-40" has received 200 kg
 When the warehouse keeper receives the remaining 100 kg against it</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>Then it still shows the state "Received"
 And a new receipt form downloads with its own form number</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr"/>
-      <c r="L28" s="3" t="inlineStr"/>
-      <c r="M28" s="3" t="inlineStr">
+      <c r="K32" s="3" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr"/>
+      <c r="M32" s="3" t="inlineStr">
         <is>
           <t>Warehouse keeper</t>
         </is>
       </c>
-      <c r="N28" s="3" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>UAT-28</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="N32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>UAT-32</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>The order closes when every line is received and invoiced</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>Received: close, to Completed</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>T5, T6</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>D9, D15</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>Given purchase order "PO-5110" is "Received"
 And the supplier's invoice for it is recorded
 When the buyer closes it</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>Then it shows the state "Completed"</t>
         </is>
       </c>
-      <c r="K29" s="3" t="inlineStr"/>
-      <c r="L29" s="3" t="inlineStr"/>
-      <c r="M29" s="3" t="inlineStr">
+      <c r="K33" s="3" t="inlineStr"/>
+      <c r="L33" s="3" t="inlineStr"/>
+      <c r="M33" s="3" t="inlineStr">
         <is>
           <t>Purchasing staff</t>
         </is>
       </c>
-      <c r="N29" s="3" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>UAT-29</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="N33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>UAT-33</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>A received purchase order cannot be cancelled</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>purchase-order</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>refused in Received: cancel</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>T5, T6</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>D9, D15</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>Given purchase order "PO-5110" is "Received"
 When the buyer tries to cancel it</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>Then the cancellation is refused
 And the buyer sees "Goods are in stock. Return them to the supplier instead."</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr"/>
-      <c r="L30" s="3" t="inlineStr"/>
-      <c r="M30" s="3" t="inlineStr">
+      <c r="K34" s="3" t="inlineStr"/>
+      <c r="L34" s="3" t="inlineStr"/>
+      <c r="M34" s="3" t="inlineStr">
         <is>
           <t>Purchasing staff</t>
         </is>
       </c>
-      <c r="N30" s="3" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>UAT-30</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="N34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>UAT-34</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>receivables</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>The invoice is raised for the issued trip, with its due date from the contract</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>sales-invoice</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>Draft: raise, to Raised</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>R9</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>T11</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>D16, D17</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" buys under contract "K-104-2" with 30-day payment terms
 And trip "TR-131" for order "SO-2060" is "Issued"
 When the accountant raises the invoice for trip "TR-131" on 2 March for 5,000.00</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>Then invoice "INV-401" shows the state "Raised"
 And its due date is 1 April</t>
         </is>
       </c>
-      <c r="K31" s="3" t="inlineStr"/>
-      <c r="L31" s="3" t="inlineStr"/>
-      <c r="M31" s="3" t="inlineStr">
+      <c r="K35" s="3" t="inlineStr"/>
+      <c r="L35" s="3" t="inlineStr"/>
+      <c r="M35" s="3" t="inlineStr">
         <is>
           <t>Accountant</t>
         </is>
       </c>
-      <c r="N31" s="3" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>UAT-31</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="N35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>UAT-35</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>receivables</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>A trip that has not been issued cannot be invoiced</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>sales-invoice</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>refused in Draft: raise before the trip is issued</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>R9</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>T11</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>D16, D17</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" buys under contract "K-104-2" with 30-day payment terms
 And trip "TR-131" for order "SO-2060" is "Issued"
@@ -2720,63 +2973,63 @@
 When the accountant tries to raise the invoice for trip "TR-132"</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>Then the invoice is refused
 And the accountant sees "Raise the invoice for goods the warehouse has issued to the trip."</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr"/>
-      <c r="L32" s="3" t="inlineStr"/>
-      <c r="M32" s="3" t="inlineStr">
+      <c r="K36" s="3" t="inlineStr"/>
+      <c r="L36" s="3" t="inlineStr"/>
+      <c r="M36" s="3" t="inlineStr">
         <is>
           <t>Accountant</t>
         </is>
       </c>
-      <c r="N32" s="3" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>UAT-32</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="N36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>UAT-36</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>receivables</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>One transfer pays the oldest invoice first</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>sales-invoice</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>Raised: record part payment, to Partly paid</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>T11, T12</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>D16, D17</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" buys under contract "K-104-2" with 30-day payment terms
 And trip "TR-131" for order "SO-2060" is "Issued"
@@ -2786,63 +3039,63 @@
 When customer "C-104" transfers 6,000.00 and the receipt is allocated</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>Then invoice "INV-401" shows the state "Paid"
 And invoice "INV-402" shows the state "Partly paid" with 2,000.00 still due</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr"/>
-      <c r="L33" s="3" t="inlineStr"/>
-      <c r="M33" s="3" t="inlineStr">
+      <c r="K37" s="3" t="inlineStr"/>
+      <c r="L37" s="3" t="inlineStr"/>
+      <c r="M37" s="3" t="inlineStr">
         <is>
           <t>Accountant</t>
         </is>
       </c>
-      <c r="N33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>UAT-33</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="N37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>UAT-37</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>receivables</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>The last payment clears the invoice</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>sales-invoice</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>Partly paid: record final payment, to Paid</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>T11, T12</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>D16, D17</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" buys under contract "K-104-2" with 30-day payment terms
 And trip "TR-131" for order "SO-2060" is "Issued"
@@ -2850,62 +3103,62 @@
 When customer "C-104" transfers 2,000.00 and the receipt is allocated</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>Then invoice "INV-402" shows the state "Paid"</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr"/>
-      <c r="L34" s="3" t="inlineStr"/>
-      <c r="M34" s="3" t="inlineStr">
+      <c r="K38" s="3" t="inlineStr"/>
+      <c r="L38" s="3" t="inlineStr"/>
+      <c r="M38" s="3" t="inlineStr">
         <is>
           <t>Accountant</t>
         </is>
       </c>
-      <c r="N34" s="3" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>UAT-34</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="N38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>UAT-38</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>receivables</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>An invoice past its due date shows in the ageing view and holds the contract</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>sales-invoice</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>in state: Raised</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>R10</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>T11, T12</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>D16, D17</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" buys under contract "K-104-2" with 30-day payment terms
 And trip "TR-131" for order "SO-2060" is "Issued"
@@ -2913,59 +3166,59 @@
 When the ageing view is run on 20 April</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>Then invoice "INV-405" shows 19 days overdue, in the 1 to 30 days column
 And contract "K-104-2" shows "On credit hold"</t>
         </is>
       </c>
-      <c r="K35" s="3" t="inlineStr"/>
-      <c r="L35" s="3" t="inlineStr"/>
-      <c r="M35" s="3" t="inlineStr"/>
-      <c r="N35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>UAT-35</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="K39" s="3" t="inlineStr"/>
+      <c r="L39" s="3" t="inlineStr"/>
+      <c r="M39" s="3" t="inlineStr"/>
+      <c r="N39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>UAT-39</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>receivables</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>A price correction is a part credit note, not an edit</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>sales-invoice</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Raised: credit in part, to Raised</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>T11, T12</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>D16, D17</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" buys under contract "K-104-2" with 30-day payment terms
 And trip "TR-131" for order "SO-2060" is "Issued"
@@ -2973,64 +3226,64 @@
 When the chief accountant issues a credit note for 300.00 against it, with the reason "agreed price correction"</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>Then invoice "INV-401" still shows the state "Raised"
 And its balance due is 4,700.00
 And the original amount of 5,000.00 is unchanged</t>
         </is>
       </c>
-      <c r="K36" s="3" t="inlineStr"/>
-      <c r="L36" s="3" t="inlineStr"/>
-      <c r="M36" s="3" t="inlineStr">
+      <c r="K40" s="3" t="inlineStr"/>
+      <c r="L40" s="3" t="inlineStr"/>
+      <c r="M40" s="3" t="inlineStr">
         <is>
           <t>Chief accountant</t>
         </is>
       </c>
-      <c r="N36" s="3" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>UAT-36</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="N40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>UAT-40</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>receivables</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>An invoice amount cannot be edited</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>sales-invoice</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>refused in Raised: edit amount</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>T11, T12</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>D16, D17</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>Given customer "C-104" buys under contract "K-104-2" with 30-day payment terms
 And trip "TR-131" for order "SO-2060" is "Issued"
@@ -3038,63 +3291,194 @@
 When the accountant tries to change its amount to 4,500.00</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>Then the change is refused
 And the accountant sees "Correct an invoice with a credit note, never by editing it."</t>
         </is>
       </c>
-      <c r="K37" s="3" t="inlineStr"/>
-      <c r="L37" s="3" t="inlineStr"/>
-      <c r="M37" s="3" t="inlineStr">
+      <c r="K41" s="3" t="inlineStr"/>
+      <c r="L41" s="3" t="inlineStr"/>
+      <c r="M41" s="3" t="inlineStr">
         <is>
           <t>Accountant</t>
         </is>
       </c>
-      <c r="N37" s="3" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>UAT-37</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="N41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>UAT-41</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>receivables</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>One transfer equal to the balance pays the invoice in full</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>sales-invoice</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Raised: record payment, to Paid</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>T11, T12</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>D16, D17</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Given customer "C-104" buys under contract "K-104-2" with 30-day payment terms
+And trip "TR-131" for order "SO-2060" is "Issued"
+Given invoice "INV-403" for 2,500.00 is "Raised"
+And its trip is confirmed delivered
+When customer "C-104" transfers 2,500.00 and the receipt is allocated</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Then invoice "INV-403" shows the state "Paid"
+And its balance due is 0.00</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr"/>
+      <c r="L42" s="3" t="inlineStr"/>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>Accountant</t>
+        </is>
+      </c>
+      <c r="N42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>UAT-42</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>receivables</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Goods returned in full are credited in full, not deleted</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>sales-invoice</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Raised: credit in full, to Credited</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>T11, T12</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>D16, D17</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Given customer "C-104" buys under contract "K-104-2" with 30-day payment terms
+And trip "TR-131" for order "SO-2060" is "Issued"
+Given invoice "INV-404" for 1,800.00 is "Raised"
+And its trip shows the state "Returned"
+When the chief accountant issues a credit note for 1,800.00 against it, with the reason "goods returned"</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Then invoice "INV-404" shows the state "Credited"
+And its balance due is 0.00
+And invoice "INV-404" can still be found and read</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr"/>
+      <c r="L43" s="3" t="inlineStr"/>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>Chief accountant</t>
+        </is>
+      </c>
+      <c r="N43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>UAT-43</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>sale-statuses</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>A new sale starts with all three statuses open</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>sale-statuses</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>in state: Not invoiced, Not delivered, Unpaid</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>T11, T17, T12</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>D8, D16, D17</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2060" for 8,000.00 ships on two trips
 And trip "TR-131" carries 5,000.00 of it and trip "TR-132" carries 3,000.00
@@ -3102,58 +3486,58 @@
 When order "SO-2060" is confirmed</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>Then its statuses are "Not invoiced", "Not delivered" and "Unpaid"</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr"/>
-      <c r="L38" s="3" t="inlineStr"/>
-      <c r="M38" s="3" t="inlineStr"/>
-      <c r="N38" s="3" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>UAT-38</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="K44" s="3" t="inlineStr"/>
+      <c r="L44" s="3" t="inlineStr"/>
+      <c r="M44" s="3" t="inlineStr"/>
+      <c r="N44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>UAT-44</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>sale-statuses</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>The first trip's invoice makes the sale partly invoiced</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>sale-statuses</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>Not invoiced: first trip invoiced, to Partly invoiced</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>T11, T17, T12</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>D8, D16, D17</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2060" for 8,000.00 ships on two trips
 And trip "TR-131" carries 5,000.00 of it and trip "TR-132" carries 3,000.00
@@ -3161,58 +3545,58 @@
 When the invoice for trip "TR-131" is raised</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>Then its statuses are "Partly invoiced", "Not delivered" and "Unpaid"</t>
         </is>
       </c>
-      <c r="K39" s="3" t="inlineStr"/>
-      <c r="L39" s="3" t="inlineStr"/>
-      <c r="M39" s="3" t="inlineStr"/>
-      <c r="N39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>UAT-39</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="K45" s="3" t="inlineStr"/>
+      <c r="L45" s="3" t="inlineStr"/>
+      <c r="M45" s="3" t="inlineStr"/>
+      <c r="N45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>UAT-45</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>sale-statuses</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Delivery never runs ahead of invoicing</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>sale-statuses</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Not delivered: first trip delivered, to Partly delivered</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>T11, T17, T12</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>D8, D16, D17</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2060" for 8,000.00 ships on two trips
 And trip "TR-131" carries 5,000.00 of it and trip "TR-132" carries 3,000.00
@@ -3221,58 +3605,58 @@
 When trip "TR-131" is confirmed delivered</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>Then its statuses are "Partly invoiced", "Partly delivered" and "Unpaid"</t>
         </is>
       </c>
-      <c r="K40" s="3" t="inlineStr"/>
-      <c r="L40" s="3" t="inlineStr"/>
-      <c r="M40" s="3" t="inlineStr"/>
-      <c r="N40" s="3" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>UAT-40</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="K46" s="3" t="inlineStr"/>
+      <c r="L46" s="3" t="inlineStr"/>
+      <c r="M46" s="3" t="inlineStr"/>
+      <c r="N46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>UAT-46</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>sale-statuses</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>A delivered sale waits on its credit terms</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>sale-statuses</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>in state: Invoiced, Delivered, Unpaid</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>R10</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>T11, T17, T12</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>D8, D16, D17</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2060" for 8,000.00 ships on two trips
 And trip "TR-131" carries 5,000.00 of it and trip "TR-132" carries 3,000.00
@@ -3281,59 +3665,59 @@
 And both trips are confirmed delivered</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
         <is>
           <t>Then its statuses are "Invoiced", "Delivered" and "Unpaid"
 And its invoices fall due on 1 April and 4 April</t>
         </is>
       </c>
-      <c r="K41" s="3" t="inlineStr"/>
-      <c r="L41" s="3" t="inlineStr"/>
-      <c r="M41" s="3" t="inlineStr"/>
-      <c r="N41" s="3" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>UAT-41</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="K47" s="3" t="inlineStr"/>
+      <c r="L47" s="3" t="inlineStr"/>
+      <c r="M47" s="3" t="inlineStr"/>
+      <c r="N47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>UAT-47</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>sale-statuses</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>A returned trip does not leave the sale waiting</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>sale-statuses</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Partly delivered: last trip delivered, to Delivered</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>T11, T17, T12</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>D8, D16, D17</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2060" for 8,000.00 ships on two trips
 And trip "TR-131" carries 5,000.00 of it and trip "TR-132" carries 3,000.00
@@ -3343,59 +3727,59 @@
 When the return is recorded</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr">
         <is>
           <t>Then its delivery status is "Delivered"
 And order "SO-2060" can complete</t>
         </is>
       </c>
-      <c r="K42" s="3" t="inlineStr"/>
-      <c r="L42" s="3" t="inlineStr"/>
-      <c r="M42" s="3" t="inlineStr"/>
-      <c r="N42" s="3" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>UAT-42</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="K48" s="3" t="inlineStr"/>
+      <c r="L48" s="3" t="inlineStr"/>
+      <c r="M48" s="3" t="inlineStr"/>
+      <c r="N48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>UAT-48</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>sale-statuses</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>A sale cannot be delivered before it is invoiced</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>sale-statuses</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>refused in Not invoiced: deliver before invoicing</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>R9</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>T11, T17, T12</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>D8, D16, D17</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr">
         <is>
           <t>Given order "SO-2060" for 8,000.00 ships on two trips
 And trip "TR-131" carries 5,000.00 of it and trip "TR-132" carries 3,000.00
@@ -3404,330 +3788,393 @@
 When a delivery is recorded for trip "TR-131"</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="J49" s="2" t="inlineStr">
         <is>
           <t>Then the delivery is refused
 And the coordinator sees "A trip leaves only with its invoice. Raise the trip's invoice first."
 And its statuses are still "Not invoiced", "Not delivered" and "Unpaid"</t>
         </is>
       </c>
-      <c r="K43" s="3" t="inlineStr"/>
-      <c r="L43" s="3" t="inlineStr"/>
-      <c r="M43" s="3" t="inlineStr">
+      <c r="K49" s="3" t="inlineStr"/>
+      <c r="L49" s="3" t="inlineStr"/>
+      <c r="M49" s="3" t="inlineStr">
         <is>
           <t>Logistics coordinator</t>
         </is>
       </c>
-      <c r="N43" s="3" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>UAT-43</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="N49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>UAT-49</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>voucher-posting</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>A saved voucher does not reach the ledger</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>voucher</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>in state: Saved</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>T12, T13</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>Given the accountant saves receipt voucher "RV-0907" for 12,400.00 from customer "C-104"
 When the ledger for customer "C-104" is read</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
         <is>
           <t>Then receipt voucher "RV-0907" is not on it</t>
         </is>
       </c>
-      <c r="K44" s="3" t="inlineStr"/>
-      <c r="L44" s="3" t="inlineStr"/>
-      <c r="M44" s="3" t="inlineStr"/>
-      <c r="N44" s="3" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>UAT-44</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="K50" s="3" t="inlineStr"/>
+      <c r="L50" s="3" t="inlineStr"/>
+      <c r="M50" s="3" t="inlineStr"/>
+      <c r="N50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>UAT-50</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>voucher-posting</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>Posting locks the voucher and updates the ledger</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>voucher</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>Saved: post, to Posted</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>T12, T13</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="I51" s="2" t="inlineStr">
         <is>
           <t>Given receipt voucher "RV-0907" is "Saved" and its entries balance
 When the accountant posts it</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="J51" s="2" t="inlineStr">
         <is>
           <t>Then it shows the state "Posted"
 And the ledger for customer "C-104" shows 12,400.00 received</t>
         </is>
       </c>
-      <c r="K45" s="3" t="inlineStr"/>
-      <c r="L45" s="3" t="inlineStr"/>
-      <c r="M45" s="3" t="inlineStr">
+      <c r="K51" s="3" t="inlineStr"/>
+      <c r="L51" s="3" t="inlineStr"/>
+      <c r="M51" s="3" t="inlineStr">
         <is>
           <t>Accountant</t>
         </is>
       </c>
-      <c r="N45" s="3" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>UAT-45</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="N51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>UAT-51</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>voucher-posting</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>A posted voucher is corrected by a reversal</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>voucher</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>Posted: reverse, to Reversed</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>T12, T13</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr">
         <is>
           <t>Given receipt voucher "RV-0907" is "Posted"
 When the chief accountant reverses it with the reason "Wrong customer"</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="J52" s="2" t="inlineStr">
         <is>
           <t>Then receipt voucher "RV-0907" shows the state "Reversed"
 And a reversing voucher for 12,400.00 is posted
 And both vouchers stay in the sequence</t>
         </is>
       </c>
-      <c r="K46" s="3" t="inlineStr"/>
-      <c r="L46" s="3" t="inlineStr"/>
-      <c r="M46" s="3" t="inlineStr">
+      <c r="K52" s="3" t="inlineStr"/>
+      <c r="L52" s="3" t="inlineStr"/>
+      <c r="M52" s="3" t="inlineStr">
         <is>
           <t>Chief accountant</t>
         </is>
       </c>
-      <c r="N46" s="3" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>UAT-46</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="N52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>UAT-52</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>voucher-posting</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>A posted voucher cannot be edited</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>voucher</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>refused in Posted: edit</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>T12, T13</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr">
+      <c r="I53" s="2" t="inlineStr">
         <is>
           <t>Given receipt voucher "RV-0907" is "Posted"
 When the accountant tries to change its amount to 12,000.00</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="J53" s="2" t="inlineStr">
         <is>
           <t>Then the change is refused
 And the accountant sees "A posted voucher is locked. Reverse it instead."</t>
         </is>
       </c>
-      <c r="K47" s="3" t="inlineStr"/>
-      <c r="L47" s="3" t="inlineStr"/>
-      <c r="M47" s="3" t="inlineStr">
+      <c r="K53" s="3" t="inlineStr"/>
+      <c r="L53" s="3" t="inlineStr"/>
+      <c r="M53" s="3" t="inlineStr">
         <is>
           <t>Accountant</t>
         </is>
       </c>
-      <c r="N47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>UAT-47</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="N53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>UAT-53</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>voucher-posting</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>A saved voucher cannot be deleted</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>voucher</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>refused in Saved: delete</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>T12, T13</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="I54" s="2" t="inlineStr">
         <is>
           <t>Given receipt voucher "RV-0911" is "Saved"
 When the accountant tries to delete it</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="J54" s="2" t="inlineStr">
         <is>
           <t>Then the deletion is refused
 And the accountant sees "Nothing is ever deleted. Void it instead."</t>
         </is>
       </c>
-      <c r="K48" s="3" t="inlineStr"/>
-      <c r="L48" s="3" t="inlineStr"/>
-      <c r="M48" s="3" t="inlineStr">
+      <c r="K54" s="3" t="inlineStr"/>
+      <c r="L54" s="3" t="inlineStr"/>
+      <c r="M54" s="3" t="inlineStr">
         <is>
           <t>Accountant</t>
         </is>
       </c>
-      <c r="N48" s="3" t="inlineStr"/>
+      <c r="N54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>UAT-54</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>voucher-posting</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>A saved voucher that is not needed is voided and keeps its number</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>voucher</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Saved: void, to Voided</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>T12, T13</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Given payment voucher "PV-0312" is "Saved"
+When the accountant voids it</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Then payment voucher "PV-0312" shows the state "Voided"
+And its amount is 0.00
+And its number stays in the sequence</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr"/>
+      <c r="L55" s="3" t="inlineStr"/>
+      <c r="M55" s="3" t="inlineStr">
+        <is>
+          <t>Accountant</t>
+        </is>
+      </c>
+      <c r="N55" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:L48">
+  <conditionalFormatting sqref="L2:L55">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3736,7 +4183,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L48" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Result" error="Choose Pass, Fail or Blocked." type="list">
+    <dataValidation sqref="L2:L55" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Result" error="Choose Pass, Fail or Blocked." type="list">
       <formula1>"Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3854,15 +4301,15 @@
         </is>
       </c>
       <c r="E2" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A2)</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A2)</f>
         <v/>
       </c>
       <c r="F2" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A2,UAT!$L$2:$L$48,"Pass")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A2,UAT!$L$2:$L$55,"Pass")</f>
         <v/>
       </c>
       <c r="G2" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A2,UAT!$L$2:$L$48,"Fail")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A2,UAT!$L$2:$L$55,"Fail")</f>
         <v/>
       </c>
       <c r="H2" s="2">
@@ -3896,15 +4343,15 @@
         </is>
       </c>
       <c r="E3" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A3)</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A3)</f>
         <v/>
       </c>
       <c r="F3" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A3,UAT!$L$2:$L$48,"Pass")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A3,UAT!$L$2:$L$55,"Pass")</f>
         <v/>
       </c>
       <c r="G3" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A3,UAT!$L$2:$L$48,"Fail")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A3,UAT!$L$2:$L$55,"Fail")</f>
         <v/>
       </c>
       <c r="H3" s="2">
@@ -3938,15 +4385,15 @@
         </is>
       </c>
       <c r="E4" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A4)</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A4)</f>
         <v/>
       </c>
       <c r="F4" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A4,UAT!$L$2:$L$48,"Pass")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A4,UAT!$L$2:$L$55,"Pass")</f>
         <v/>
       </c>
       <c r="G4" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A4,UAT!$L$2:$L$48,"Fail")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A4,UAT!$L$2:$L$55,"Fail")</f>
         <v/>
       </c>
       <c r="H4" s="2">
@@ -3980,15 +4427,15 @@
         </is>
       </c>
       <c r="E5" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A5)</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A5)</f>
         <v/>
       </c>
       <c r="F5" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A5,UAT!$L$2:$L$48,"Pass")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A5,UAT!$L$2:$L$55,"Pass")</f>
         <v/>
       </c>
       <c r="G5" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A5,UAT!$L$2:$L$48,"Fail")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A5,UAT!$L$2:$L$55,"Fail")</f>
         <v/>
       </c>
       <c r="H5" s="2">
@@ -4022,15 +4469,15 @@
         </is>
       </c>
       <c r="E6" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A6)</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A6)</f>
         <v/>
       </c>
       <c r="F6" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A6,UAT!$L$2:$L$48,"Pass")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A6,UAT!$L$2:$L$55,"Pass")</f>
         <v/>
       </c>
       <c r="G6" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A6,UAT!$L$2:$L$48,"Fail")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A6,UAT!$L$2:$L$55,"Fail")</f>
         <v/>
       </c>
       <c r="H6" s="2">
@@ -4064,15 +4511,15 @@
         </is>
       </c>
       <c r="E7" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A7)</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A7)</f>
         <v/>
       </c>
       <c r="F7" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A7,UAT!$L$2:$L$48,"Pass")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A7,UAT!$L$2:$L$55,"Pass")</f>
         <v/>
       </c>
       <c r="G7" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A7,UAT!$L$2:$L$48,"Fail")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A7,UAT!$L$2:$L$55,"Fail")</f>
         <v/>
       </c>
       <c r="H7" s="2">
@@ -4106,15 +4553,15 @@
         </is>
       </c>
       <c r="E8" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A8)</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A8)</f>
         <v/>
       </c>
       <c r="F8" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A8,UAT!$L$2:$L$48,"Pass")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A8,UAT!$L$2:$L$55,"Pass")</f>
         <v/>
       </c>
       <c r="G8" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A8,UAT!$L$2:$L$48,"Fail")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A8,UAT!$L$2:$L$55,"Fail")</f>
         <v/>
       </c>
       <c r="H8" s="2">
@@ -4148,15 +4595,15 @@
         </is>
       </c>
       <c r="E9" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A9)</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A9)</f>
         <v/>
       </c>
       <c r="F9" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A9,UAT!$L$2:$L$48,"Pass")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A9,UAT!$L$2:$L$55,"Pass")</f>
         <v/>
       </c>
       <c r="G9" s="2">
-        <f>COUNTIFS(UAT!$B$2:$B$48,A9,UAT!$L$2:$L$48,"Fail")</f>
+        <f>COUNTIFS(UAT!$B$2:$B$55,A9,UAT!$L$2:$L$55,"Fail")</f>
         <v/>
       </c>
       <c r="H9" s="2">
@@ -4187,7 +4634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4236,7 +4683,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>UAT-17, UAT-18, UAT-19, UAT-20, UAT-21, UAT-22, UAT-30, UAT-31, UAT-32, UAT-33, UAT-34, UAT-35, UAT-36, UAT-37, UAT-38, UAT-39, UAT-40, UAT-41, UAT-42, UAT-43, UAT-44</t>
+          <t>UAT-21, UAT-22, UAT-23, UAT-24, UAT-25, UAT-26, UAT-34, UAT-35, UAT-36, UAT-37, UAT-38, UAT-39, UAT-40, UAT-41, UAT-42, UAT-43, UAT-44, UAT-45, UAT-46, UAT-47, UAT-48, UAT-49, UAT-50</t>
         </is>
       </c>
     </row>
@@ -4258,7 +4705,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>UAT-19, UAT-20, UAT-30, UAT-31, UAT-32, UAT-33, UAT-34, UAT-35, UAT-36, UAT-37, UAT-38, UAT-39, UAT-40, UAT-41, UAT-42</t>
+          <t>UAT-23, UAT-24, UAT-34, UAT-35, UAT-36, UAT-37, UAT-38, UAT-39, UAT-40, UAT-41, UAT-42, UAT-43, UAT-44, UAT-45, UAT-46, UAT-47, UAT-48</t>
         </is>
       </c>
     </row>
@@ -4275,12 +4722,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>In transit, Issued, Planned</t>
+          <t>Delivered, In transit, Issued, Planned</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>UAT-01, UAT-02, UAT-03, UAT-04, UAT-05, UAT-06</t>
+          <t>UAT-01, UAT-02, UAT-03, UAT-04, UAT-05, UAT-06, UAT-07</t>
         </is>
       </c>
     </row>
@@ -4302,7 +4749,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>UAT-30, UAT-31, UAT-32, UAT-33, UAT-34, UAT-35, UAT-36, UAT-37, UAT-38, UAT-39, UAT-40, UAT-41, UAT-42</t>
+          <t>UAT-34, UAT-35, UAT-36, UAT-37, UAT-38, UAT-39, UAT-40, UAT-41, UAT-42, UAT-43, UAT-44, UAT-45, UAT-46, UAT-47, UAT-48</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4771,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>UAT-31, UAT-37, UAT-38, UAT-39, UAT-40, UAT-41, UAT-42</t>
+          <t>UAT-35, UAT-43, UAT-44, UAT-45, UAT-46, UAT-47, UAT-48</t>
         </is>
       </c>
     </row>
@@ -4346,7 +4793,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>UAT-07, UAT-08, UAT-09, UAT-10, UAT-11, UAT-12</t>
+          <t>UAT-08, UAT-09, UAT-10, UAT-11, UAT-12, UAT-13</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4815,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>UAT-12</t>
+          <t>UAT-13</t>
         </is>
       </c>
     </row>
@@ -4390,7 +4837,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>UAT-23, UAT-24, UAT-25, UAT-26, UAT-28, UAT-29</t>
+          <t>UAT-27, UAT-28, UAT-29, UAT-30, UAT-32, UAT-33</t>
         </is>
       </c>
     </row>
@@ -4412,7 +4859,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>UAT-27</t>
+          <t>UAT-31</t>
         </is>
       </c>
     </row>
@@ -4456,7 +4903,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>UAT-30, UAT-32, UAT-35, UAT-36</t>
+          <t>UAT-34, UAT-36, UAT-39, UAT-40</t>
         </is>
       </c>
     </row>
@@ -4478,14 +4925,14 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>UAT-32, UAT-33</t>
+          <t>UAT-36, UAT-37</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>INV-405</t>
+          <t>INV-403</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -4500,58 +4947,58 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>UAT-34</t>
+          <t>UAT-41</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SO-2031</t>
+          <t>INV-404</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>sales order</t>
+          <t>sales invoice</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Open, With logistics</t>
+          <t>Raised</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>UAT-21, UAT-22</t>
+          <t>UAT-42</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>SO-2040</t>
+          <t>INV-405</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>sales order</t>
+          <t>sales invoice</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Cancelled, Open</t>
+          <t>Raised</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>UAT-13, UAT-15</t>
+          <t>UAT-38</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>SO-2041</t>
+          <t>SO-2031</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -4561,19 +5008,19 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>In production</t>
+          <t>Open, With logistics</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>UAT-14, UAT-16</t>
+          <t>UAT-25, UAT-26</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>SO-2050</t>
+          <t>SO-2040</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -4583,19 +5030,19 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Receiving and shipping</t>
+          <t>Cancelled, Open</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>UAT-01, UAT-02, UAT-03, UAT-04, UAT-05, UAT-06</t>
+          <t>UAT-14, UAT-16</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>SO-2060</t>
+          <t>SO-2041</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -4605,19 +5052,19 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>as the row's steps say</t>
+          <t>In production</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>UAT-30, UAT-31, UAT-32, UAT-33, UAT-34, UAT-35, UAT-36, UAT-37, UAT-38, UAT-39, UAT-40, UAT-41, UAT-42</t>
+          <t>UAT-15, UAT-17</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>SO-2070</t>
+          <t>SO-2043</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -4627,34 +5074,122 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>In production</t>
+          <t>Receiving and shipping</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>UAT-07, UAT-08, UAT-09, UAT-10, UAT-11, UAT-12</t>
+          <t>UAT-18, UAT-19</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>SO-2044</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>sales order</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>UAT-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>SO-2050</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>sales order</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Receiving and shipping</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>UAT-01, UAT-02, UAT-03, UAT-04, UAT-05, UAT-06, UAT-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>SO-2060</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>sales order</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>as the row's steps say</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>UAT-34, UAT-35, UAT-36, UAT-37, UAT-38, UAT-39, UAT-40, UAT-41, UAT-42, UAT-43, UAT-44, UAT-45, UAT-46, UAT-47, UAT-48</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>SO-2070</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>sales order</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>In production</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>UAT-08, UAT-09, UAT-10, UAT-11, UAT-12, UAT-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>V-07</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>as the row's steps say</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>UAT-23</t>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>UAT-27</t>
         </is>
       </c>
     </row>
@@ -4744,7 +5279,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr"/>
       <c r="C2" s="2">
-        <f>IF(B2="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B2,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B2="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B2,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D2" s="3" t="inlineStr"/>
@@ -4763,7 +5298,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr"/>
       <c r="C3" s="2">
-        <f>IF(B3="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B3,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B3="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B3,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D3" s="3" t="inlineStr"/>
@@ -4782,7 +5317,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr"/>
       <c r="C4" s="2">
-        <f>IF(B4="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B4,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B4="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B4,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D4" s="3" t="inlineStr"/>
@@ -4801,7 +5336,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr"/>
       <c r="C5" s="2">
-        <f>IF(B5="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B5,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B5="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B5,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D5" s="3" t="inlineStr"/>
@@ -4820,7 +5355,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr"/>
       <c r="C6" s="2">
-        <f>IF(B6="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B6,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B6="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B6,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D6" s="3" t="inlineStr"/>
@@ -4839,7 +5374,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr"/>
       <c r="C7" s="2">
-        <f>IF(B7="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B7,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B7="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B7,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D7" s="3" t="inlineStr"/>
@@ -4858,7 +5393,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr"/>
       <c r="C8" s="2">
-        <f>IF(B8="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B8,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B8="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B8,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D8" s="3" t="inlineStr"/>
@@ -4877,7 +5412,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr"/>
       <c r="C9" s="2">
-        <f>IF(B9="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B9,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B9="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B9,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D9" s="3" t="inlineStr"/>
@@ -4896,7 +5431,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr"/>
       <c r="C10" s="2">
-        <f>IF(B10="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B10,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B10="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B10,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D10" s="3" t="inlineStr"/>
@@ -4915,7 +5450,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr"/>
       <c r="C11" s="2">
-        <f>IF(B11="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B11,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B11="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B11,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D11" s="3" t="inlineStr"/>
@@ -4934,7 +5469,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr"/>
       <c r="C12" s="2">
-        <f>IF(B12="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B12,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B12="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B12,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D12" s="3" t="inlineStr"/>
@@ -4953,7 +5488,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr"/>
       <c r="C13" s="2">
-        <f>IF(B13="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B13,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B13="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B13,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -4972,7 +5507,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr"/>
       <c r="C14" s="2">
-        <f>IF(B14="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B14,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B14="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B14,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D14" s="3" t="inlineStr"/>
@@ -4991,7 +5526,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr"/>
       <c r="C15" s="2">
-        <f>IF(B15="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B15,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B15="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B15,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D15" s="3" t="inlineStr"/>
@@ -5010,7 +5545,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr"/>
       <c r="C16" s="2">
-        <f>IF(B16="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B16,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B16="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B16,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D16" s="3" t="inlineStr"/>
@@ -5029,7 +5564,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr"/>
       <c r="C17" s="2">
-        <f>IF(B17="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B17,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B17="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B17,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D17" s="3" t="inlineStr"/>
@@ -5048,7 +5583,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr"/>
       <c r="C18" s="2">
-        <f>IF(B18="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B18,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B18="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B18,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D18" s="3" t="inlineStr"/>
@@ -5067,7 +5602,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr"/>
       <c r="C19" s="2">
-        <f>IF(B19="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B19,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B19="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B19,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D19" s="3" t="inlineStr"/>
@@ -5086,7 +5621,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr"/>
       <c r="C20" s="2">
-        <f>IF(B20="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B20,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B20="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B20,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D20" s="3" t="inlineStr"/>
@@ -5105,7 +5640,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr"/>
       <c r="C21" s="2">
-        <f>IF(B21="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B21,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B21="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B21,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D21" s="3" t="inlineStr"/>
@@ -5124,7 +5659,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr"/>
       <c r="C22" s="2">
-        <f>IF(B22="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B22,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B22="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B22,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D22" s="3" t="inlineStr"/>
@@ -5143,7 +5678,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr"/>
       <c r="C23" s="2">
-        <f>IF(B23="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B23,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B23="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B23,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D23" s="3" t="inlineStr"/>
@@ -5162,7 +5697,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr"/>
       <c r="C24" s="2">
-        <f>IF(B24="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B24,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B24="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B24,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D24" s="3" t="inlineStr"/>
@@ -5181,7 +5716,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr"/>
       <c r="C25" s="2">
-        <f>IF(B25="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B25,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B25="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B25,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D25" s="3" t="inlineStr"/>
@@ -5200,7 +5735,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr"/>
       <c r="C26" s="2">
-        <f>IF(B26="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B26,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B26="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B26,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D26" s="3" t="inlineStr"/>
@@ -5219,7 +5754,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr"/>
       <c r="C27" s="2">
-        <f>IF(B27="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B27,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B27="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B27,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D27" s="3" t="inlineStr"/>
@@ -5238,7 +5773,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr"/>
       <c r="C28" s="2">
-        <f>IF(B28="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B28,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B28="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B28,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D28" s="3" t="inlineStr"/>
@@ -5257,7 +5792,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr"/>
       <c r="C29" s="2">
-        <f>IF(B29="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B29,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B29="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B29,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D29" s="3" t="inlineStr"/>
@@ -5276,7 +5811,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr"/>
       <c r="C30" s="2">
-        <f>IF(B30="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B30,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B30="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B30,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D30" s="3" t="inlineStr"/>
@@ -5295,7 +5830,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr"/>
       <c r="C31" s="2">
-        <f>IF(B31="","",IFERROR(INDEX(UAT!$B$2:$B$48,MATCH(B31,UAT!$A$2:$A$48,0)),"not a UAT row"))</f>
+        <f>IF(B31="","",IFERROR(INDEX(UAT!$B$2:$B$55,MATCH(B31,UAT!$A$2:$A$55,0)),"not a UAT row"))</f>
         <v/>
       </c>
       <c r="D31" s="3" t="inlineStr"/>
@@ -5309,7 +5844,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="B2:B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="UAT row" error="Choose from the list." type="list">
-      <formula1>=UAT!$A$2:$A$48</formula1>
+      <formula1>=UAT!$A$2:$A$55</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Severity" error="Choose from the list." type="list">
       <formula1>"1,2,3"</formula1>

</xml_diff>